<commit_message>
docs: complete N5 N6 literature extraction
</commit_message>
<xml_diff>
--- a/文献综述/03_静态创新专项/泛式/P02_泛式文献证据矩阵.xlsx
+++ b/文献综述/03_静态创新专项/泛式/P02_泛式文献证据矩阵.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Scope" sheetId="1" r:id="R98d833f02417478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="2" r:id="Rac2b3ef036194e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="3" r:id="R611beec1580b4919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim Map" sheetId="4" r:id="Rda23af1342614aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparability" sheetId="5" r:id="R29e6219765f54fd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unresolved" sheetId="6" r:id="R4ea870fcfa7649c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Log" sheetId="7" r:id="R6939c34a67854960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Scope" sheetId="1" r:id="R53bcb920888f4b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="2" r:id="R72824c4f1a0b4607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="3" r:id="R533f956437184f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claim Map" sheetId="4" r:id="Rb0a3ad022bd54734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparability" sheetId="5" r:id="Rcb77f651e337431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unresolved" sheetId="6" r:id="R634c6953f1004dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Log" sheetId="7" r:id="R32a1a3d487624c60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1126,7 +1126,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6af6270f7174e73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb854da6b5a784746"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2146,7 +2146,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c5d9ffe08349c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfaa53e09ae54dc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2499,7 +2499,7 @@
         <x:v>L001</x:v>
       </x:c>
       <x:c r="C4" s="27" t="str">
-        <x:v>B001；直接：Abstract；`three types of disturbances`；`event-driven rescheduling`；模型与编码章节</x:v>
+        <x:v>B001 `5.1 Encoding and decoding`、Algorithms 5–6、`6.4`–`6.5`；B001 `6.1`–`6.5`</x:v>
       </x:c>
       <x:c r="D4" s="27" t="str">
         <x:v>Verified</x:v>
@@ -2565,64 +2565,64 @@
         <x:v>核心研究对象；原分类=混合；动/确</x:v>
       </x:c>
       <x:c r="Y4" s="27" t="str">
-        <x:v>QNSGA-II：混合初始化＋NSGA-II＋Q-learning选择N1–N6；事件驱动IS/RS/CS重调度</x:v>
+        <x:v>OS–MS–AS 三段染色体</x:v>
       </x:c>
       <x:c r="Z4" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>电量检查→充电→机器最早可行空档左移插入</x:v>
       </x:c>
       <x:c r="AA4" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>编码保持可行，无复杂染色体修复</x:v>
       </x:c>
       <x:c r="AB4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>与对照统一 CPU 时间；动态重调度为初始调度时间的一半</x:v>
       </x:c>
       <x:c r="AC4" s="27" t="str">
-        <x:v>QNSGA-II：混合初始化＋NSGA-II＋Q-learning选择N1–N6；事件驱动IS/RS/CS重调度</x:v>
+        <x:v>混合初始化→NSGA-II；环境状态驱动 Q-learning 在 N1–N6 中选邻域，局部搜索嵌入每代进化</x:v>
       </x:c>
       <x:c r="AD4" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>混合初始化→NSGA-II；环境状态驱动 Q-learning 在 N1–N6 中选邻域，局部搜索嵌入每代进化</x:v>
       </x:c>
       <x:c r="AE4" s="27" t="str">
-        <x:v>扩展Brandimarte；HV/IGD/C-metric；完整预算与重复协议待P02/N6映射</x:v>
+        <x:v>扩展Brandimarte的EMK01–EMK10；10/15/20工件，3/4/5 AGV</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>10/15/20</x:v>
       </x:c>
       <x:c r="AG4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>随Brandimarte实例</x:v>
       </x:c>
       <x:c r="AH4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见EMK实例</x:v>
       </x:c>
       <x:c r="AI4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>3/4/5</x:v>
       </x:c>
       <x:c r="AJ4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>原MK布局与运输矩阵</x:v>
       </x:c>
       <x:c r="AK4" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>三档</x:v>
       </x:c>
       <x:c r="AL4" s="27" t="str">
-        <x:v>QNSGA-II消融与三算法比较</x:v>
+        <x:v>消融A/B/C；NSGA-II、MOEA/D、MOPSO；IS/RS/CS</x:v>
       </x:c>
       <x:c r="AM4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>N=100；比较算法CPU时间相同；重调度时间为初始的一半</x:v>
       </x:c>
       <x:c r="AN4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>N=100；比较算法CPU时间相同；重调度时间为初始的一半</x:v>
       </x:c>
       <x:c r="AO4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="AP4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ4" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>Taguchi L9参数试验；结果以均值/箱线图报告</x:v>
       </x:c>
       <x:c r="AR4" s="27" t="str">
-        <x:v>效率；能源；稳定性；多目标组合</x:v>
+        <x:v>makespan、TEC、HV、IGD（各算法非支配并集替代真PF）、C-metric、RSI及MCR/σa/APSD</x:v>
       </x:c>
       <x:c r="AS4" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -2634,13 +2634,13 @@
         <x:v>直接：Abstract；`three types of disturbances`；`event-driven rescheduling`；模型与编码章节；扩展Brandimarte；HV/IGD/C-metric；完整预算与重复协议待P02/N6映射</x:v>
       </x:c>
       <x:c r="AV4" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B001 `5.1 Encoding and decoding`、Algorithms 5–6、`6.4`–`6.5`；B001 `6.1`–`6.5`</x:v>
       </x:c>
       <x:c r="AW4" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX4" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY4" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -2649,7 +2649,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA4" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB4" s="27" t="str">
         <x:v>OK</x:v>
@@ -2663,7 +2663,7 @@
         <x:v>L002</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
-        <x:v>B002；直接：摘要；`FJSP-AGV`；“不同编码段”；“最大完工时间”</x:v>
+        <x:v>B002 `2.1 算法整体流程`、`2.2`、`2.3`、图7；B002 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
         <x:v>Verified</x:v>
@@ -2729,64 +2729,64 @@
         <x:v>核心车间原始研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y5" s="27" t="str">
-        <x:v>FJSP–AGV静态混合求解；不同编码段与AGV数量约束（具体优化器待N5精读）</x:v>
+        <x:v>OS–MS–AS 三层工序编码</x:v>
       </x:c>
       <x:c r="Z5" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>遍历机器可用时间并插入最早满足约束的空档</x:v>
       </x:c>
       <x:c r="AA5" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>OS 邻域变异后按相同位置同步调整 MS；POX/PBX 保持段内可行</x:v>
       </x:c>
       <x:c r="AB5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>100 代</x:v>
       </x:c>
       <x:c r="AC5" s="27" t="str">
-        <x:v>FJSP–AGV静态混合求解；不同编码段与AGV数量约束（具体优化器待N5精读）</x:v>
+        <x:v>80%随机+20%启发式初始化→选择/交叉/变异→外部精英库；停滞时启发式引导变异</x:v>
       </x:c>
       <x:c r="AD5" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>80%随机+20%启发式初始化→选择/交叉/变异→外部精英库；停滞时启发式引导变异</x:v>
       </x:c>
       <x:c r="AE5" s="27" t="str">
-        <x:v>静态FJSP–AGV算例；规模、重复和统计待N6抽取</x:v>
+        <x:v>Deroussi 10例：5–8工件、2–5工序、8机器、2AGV；EX布局例：可选3机器、4布局、3AGV</x:v>
       </x:c>
       <x:c r="AF5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>5–8（数据集1）</x:v>
       </x:c>
       <x:c r="AG5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>每工件2–5（数据集1）</x:v>
       </x:c>
       <x:c r="AH5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>8（数据集1）</x:v>
       </x:c>
       <x:c r="AI5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>2（数据集1）；3（数据集2）</x:v>
       </x:c>
       <x:c r="AJ5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>4种布局（数据集2）</x:v>
       </x:c>
       <x:c r="AK5" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>中小规模</x:v>
       </x:c>
       <x:c r="AL5" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>GA、IGA及文内先进算法</x:v>
       </x:c>
       <x:c r="AM5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=100，maxgen=100</x:v>
       </x:c>
       <x:c r="AN5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=100，maxgen=100</x:v>
       </x:c>
       <x:c r="AO5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ5" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR5" s="27" t="str">
-        <x:v>效率</x:v>
+        <x:v>makespan Best/Mean</x:v>
       </x:c>
       <x:c r="AS5" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -2798,13 +2798,13 @@
         <x:v>直接：摘要；`FJSP-AGV`；“不同编码段”；“最大完工时间”；静态FJSP–AGV算例；规模、重复和统计待N6抽取</x:v>
       </x:c>
       <x:c r="AV5" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B002 `2.1 算法整体流程`、`2.2`、`2.3`、图7；B002 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="AW5" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX5" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY5" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -2813,7 +2813,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA5" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB5" s="27" t="str">
         <x:v>OK</x:v>
@@ -2827,7 +2827,7 @@
         <x:v>L003</x:v>
       </x:c>
       <x:c r="C6" s="27" t="str">
-        <x:v>B003；直接：摘要“离散动态特性”“实时动态调度”；限制：具体随机模型与场景未报告</x:v>
+        <x:v>B003 `2.3 学习算法`、`5 仿真研究`；B003 `5 仿真研究`、表1</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -2893,64 +2893,64 @@
         <x:v>路径/任务相邻研究；原分类=学习型；动/未报</x:v>
       </x:c>
       <x:c r="Y6" s="27" t="str">
-        <x:v>递阶强化学习多智能体AGV调度</x:v>
+        <x:v>MaxQ 子任务状态；状态含 AGV位置/载荷、缓冲区、加工与零件到达</x:v>
       </x:c>
       <x:c r="Z6" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>基本动作执行后观察新状态与奖励，递阶更新完成函数</x:v>
       </x:c>
       <x:c r="AA6" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>对到达非目标终止状态的子策略增加负奖励</x:v>
       </x:c>
       <x:c r="AB6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>到达各子任务终止状态集</x:v>
       </x:c>
       <x:c r="AC6" s="27" t="str">
-        <x:v>递阶强化学习多智能体AGV调度</x:v>
+        <x:v>从根任务递阶展开到基本动作；局部策略更新后向上级传递完成函数</x:v>
       </x:c>
       <x:c r="AD6" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>从根任务递阶展开到基本动作；局部策略更新后向上级传递完成函数</x:v>
       </x:c>
       <x:c r="AE6" s="27" t="str">
-        <x:v>多智能体AGV实验；具体场景和随机协议未报告</x:v>
+        <x:v>图2离散事件AGV系统；20位置点、9种载荷状态及缓冲/到达状态</x:v>
       </x:c>
       <x:c r="AF6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AG6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AH6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>加工台数量见图2/表1</x:v>
       </x:c>
       <x:c r="AI6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>多AGV，数量未报告</x:v>
       </x:c>
       <x:c r="AJ6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>20个AGV位置点</x:v>
       </x:c>
       <x:c r="AK6" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>案例仿真</x:v>
       </x:c>
       <x:c r="AL6" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>启发式/无学习策略对照信息不完整</x:v>
       </x:c>
       <x:c r="AM6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>学习参数见表1；明确总训练预算未报告</x:v>
       </x:c>
       <x:c r="AN6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>学习参数见表1；明确总训练预算未报告</x:v>
       </x:c>
       <x:c r="AO6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ6" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR6" s="27" t="str">
-        <x:v>效率；未报告</x:v>
+        <x:v>累积奖励、调度/运输性能</x:v>
       </x:c>
       <x:c r="AS6" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -2962,13 +2962,13 @@
         <x:v>直接：摘要“离散动态特性”“实时动态调度”；限制：具体随机模型与场景未报告；多智能体AGV实验；具体场景和随机协议未报告</x:v>
       </x:c>
       <x:c r="AV6" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B003 `2.3 学习算法`、`5 仿真研究`；B003 `5 仿真研究`、表1</x:v>
       </x:c>
       <x:c r="AW6" s="27" t="str">
         <x:v>随机性/事件生成机制不完整</x:v>
       </x:c>
       <x:c r="AX6" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY6" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -2977,7 +2977,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA6" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB6" s="27" t="str">
         <x:v>OK</x:v>
@@ -2991,7 +2991,7 @@
         <x:v>L004</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
-        <x:v>B004；直接：摘要“异构图状态”“联合动作空间”“协同决策”</x:v>
+        <x:v>B004 `3 算法`、`4.1 实验设置`；B004 `4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>Verified</x:v>
@@ -3057,64 +3057,64 @@
         <x:v>核心车间原始研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y7" s="27" t="str">
-        <x:v>异构图注意力＋联合动作空间的学习型协同调度</x:v>
+        <x:v>异构图状态；工序、机器、AGV节点及关系；联合动作</x:v>
       </x:c>
       <x:c r="Z7" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>动作选择后更新工序加工与 AGV运输状态</x:v>
       </x:c>
       <x:c r="AA7" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>可行动作掩码/约束筛除不可执行联合动作</x:v>
       </x:c>
       <x:c r="AB7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>回合完成全部工序；训练预算见原文实验设置</x:v>
       </x:c>
       <x:c r="AC7" s="27" t="str">
-        <x:v>异构图注意力＋联合动作空间的学习型协同调度</x:v>
+        <x:v>异构图注意力编码→联合策略输出→环境推进→策略梯度更新；注意力与联合动作空间是核心插入点</x:v>
       </x:c>
       <x:c r="AD7" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>异构图注意力编码→联合策略输出→环境推进→策略梯度更新；注意力与联合动作空间是核心插入点</x:v>
       </x:c>
       <x:c r="AE7" s="27" t="str">
-        <x:v>静态联合调度实验；稳定性/鲁棒性协议待N6抽取</x:v>
+        <x:v>合成FJSP-AGV不同规模算例</x:v>
       </x:c>
       <x:c r="AF7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见合成算例表</x:v>
       </x:c>
       <x:c r="AG7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见合成算例表</x:v>
       </x:c>
       <x:c r="AH7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见合成算例表</x:v>
       </x:c>
       <x:c r="AI7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见合成算例表</x:v>
       </x:c>
       <x:c r="AJ7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AK7" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多规模</x:v>
       </x:c>
       <x:c r="AL7" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>规则、传统DRL及消融对照（以原文表为准）</x:v>
       </x:c>
       <x:c r="AM7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>超参数与训练设置见§4.1；统一停止口径未报告</x:v>
       </x:c>
       <x:c r="AN7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>超参数与训练设置见§4.1；统一停止口径未报告</x:v>
       </x:c>
       <x:c r="AO7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ7" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR7" s="27" t="str">
-        <x:v>效率；稳定性；鲁棒性</x:v>
+        <x:v>makespan、综合目标、稳定/鲁棒表现</x:v>
       </x:c>
       <x:c r="AS7" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3126,13 +3126,13 @@
         <x:v>直接：摘要“异构图状态”“联合动作空间”“协同决策”；静态联合调度实验；稳定性/鲁棒性协议待N6抽取</x:v>
       </x:c>
       <x:c r="AV7" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B004 `3 算法`、`4.1 实验设置`；B004 `4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="AW7" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX7" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY7" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3141,7 +3141,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA7" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB7" s="27" t="str">
         <x:v>OK</x:v>
@@ -3155,7 +3155,7 @@
         <x:v>L005</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
-        <x:v>B005；直接：摘要“异构AGV”“资源配置优化模型”“三层编码”</x:v>
+        <x:v>B005 `2.2 编码`、`2.3 解码`、邻域结构、`3.1`；B005 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -3221,64 +3221,64 @@
         <x:v>核心车间原始研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y8" s="27" t="str">
-        <x:v>Q-learning改进果蝇算法；三层编码；异构AGV资源配置</x:v>
+        <x:v>任务排序–AGV分配–AGV数量三层编码</x:v>
       </x:c>
       <x:c r="Z8" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>顺序解码任务与车辆分配并计算最大完工时间</x:v>
       </x:c>
       <x:c r="AA8" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>邻域生成后按问题约束保留有效任务序列/车辆层</x:v>
       </x:c>
       <x:c r="AB8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>200 代</x:v>
       </x:c>
       <x:c r="AC8" s="27" t="str">
-        <x:v>Q-learning改进果蝇算法；三层编码；异构AGV资源配置</x:v>
+        <x:v>FOA嗅觉/视觉搜索；Q-learning在 N1–N5 中选邻域，初始化与种群合并分别嵌入初始化和视觉阶段</x:v>
       </x:c>
       <x:c r="AD8" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>FOA嗅觉/视觉搜索；Q-learning在 N1–N5 中选邻域，初始化与种群合并分别嵌入初始化和视觉阶段</x:v>
       </x:c>
       <x:c r="AE8" s="27" t="str">
-        <x:v>针织车间资源配置实验；卷期与完整协议待更新</x:v>
+        <x:v>自建27例；25/50/100工件，5/25/50机器，2/10/16 AGV，3工序、2类AGV</x:v>
       </x:c>
       <x:c r="AF8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>25/50/100</x:v>
       </x:c>
       <x:c r="AG8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>每工件3</x:v>
       </x:c>
       <x:c r="AH8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>5/25/50</x:v>
       </x:c>
       <x:c r="AI8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>2/10/16（2类）</x:v>
       </x:c>
       <x:c r="AJ8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>针织车间运输时间矩阵</x:v>
       </x:c>
       <x:c r="AK8" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>三档；27例</x:v>
       </x:c>
       <x:c r="AL8" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>FOA-1/FOA-2消融；FOA、IGA、IGWO、IPSO、IABC、QABC</x:v>
       </x:c>
       <x:c r="AM8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=200，200代；ε=.8、γ=.6、α=.2</x:v>
       </x:c>
       <x:c r="AN8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=200，200代；ε=.8、γ=.6、α=.2</x:v>
       </x:c>
       <x:c r="AO8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="AP8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ8" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR8" s="27" t="str">
-        <x:v>效率；稳定性</x:v>
+        <x:v>min、avg、RPD、箱线图/收敛曲线</x:v>
       </x:c>
       <x:c r="AS8" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3290,13 +3290,13 @@
         <x:v>直接：摘要“异构AGV”“资源配置优化模型”“三层编码”；针织车间资源配置实验；卷期与完整协议待更新</x:v>
       </x:c>
       <x:c r="AV8" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B005 `2.2 编码`、`2.3 解码`、邻域结构、`3.1`；B005 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="AW8" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX8" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY8" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3305,7 +3305,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA8" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB8" s="27" t="str">
         <x:v>OK</x:v>
@@ -3319,7 +3319,7 @@
         <x:v>L006</x:v>
       </x:c>
       <x:c r="C9" s="27" t="str">
-        <x:v>B006；直接：摘要；“关键技术”；第3章；不作单一实验情境编码</x:v>
+        <x:v>B006 第3章、`5 结论与展望`；B006 第3章</x:v>
       </x:c>
       <x:c r="D9" s="27" t="str">
         <x:v>Verified</x:v>
@@ -3385,64 +3385,64 @@
         <x:v>综述；原分类=跨类型（综述）；跨/跨</x:v>
       </x:c>
       <x:c r="Y9" s="27" t="str">
-        <x:v>综述：任务数据库、路径规划、多机协同和动态管控方法</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="Z9" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AA9" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>综述归纳路径规划、多机协同、动态管控中的冲突处理</x:v>
       </x:c>
       <x:c r="AB9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AC9" s="27" t="str">
-        <x:v>综述：任务数据库、路径规划、多机协同和动态管控方法</x:v>
+        <x:v>任务数据库→路径规划→多机协同→动态管控→管理系统，为技术链而非单一优化器</x:v>
       </x:c>
       <x:c r="AD9" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>任务数据库→路径规划→多机协同→动态管控→管理系统，为技术链而非单一优化器</x:v>
       </x:c>
       <x:c r="AE9" s="27" t="str">
-        <x:v>综述，无统一实验协议</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AF9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AG9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AH9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AI9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AJ9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>跨场景</x:v>
       </x:c>
       <x:c r="AK9" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>综述</x:v>
       </x:c>
       <x:c r="AL9" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AM9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AN9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AO9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AP9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AQ9" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AR9" s="27" t="str">
-        <x:v>跨类型（综述）</x:v>
+        <x:v>无统一实验指标</x:v>
       </x:c>
       <x:c r="AS9" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3454,13 +3454,13 @@
         <x:v>直接：摘要；“关键技术”；第3章；不作单一实验情境编码；综述，无统一实验协议</x:v>
       </x:c>
       <x:c r="AV9" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B006 第3章、`5 结论与展望`；B006 第3章</x:v>
       </x:c>
       <x:c r="AW9" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX9" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6字段已完成原文深度抽取</x:v>
       </x:c>
       <x:c r="AY9" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3469,7 +3469,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA9" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB9" s="27" t="str">
         <x:v>OK</x:v>
@@ -3483,7 +3483,7 @@
         <x:v>L007</x:v>
       </x:c>
       <x:c r="C10" s="27" t="str">
-        <x:v>B007；直接：摘要/关键词；“两阶段算法”；“碰撞检测与避免”；“480”</x:v>
+        <x:v>B007 `2.2`、`3 AGV碰撞检测及避免算法`；B007 `4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>Verified</x:v>
@@ -3549,64 +3549,64 @@
         <x:v>路径/任务相邻研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y10" s="27" t="str">
-        <x:v>两阶段任务分配—路径规划＋碰撞检测/避免</x:v>
+        <x:v>运输任务、AGV与有向路网状态</x:v>
       </x:c>
       <x:c r="Z10" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>先按时间优先级分配任务，再生成路径</x:v>
       </x:c>
       <x:c r="AA10" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>时空占用检测；等待/改道消除节点与相向冲突</x:v>
       </x:c>
       <x:c r="AB10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>全部任务完成</x:v>
       </x:c>
       <x:c r="AC10" s="27" t="str">
-        <x:v>两阶段任务分配—路径规划＋碰撞检测/避免</x:v>
+        <x:v>两阶段任务分配→路径规划→碰撞检测与避免</x:v>
       </x:c>
       <x:c r="AD10" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>两阶段任务分配→路径规划→碰撞检测与避免</x:v>
       </x:c>
       <x:c r="AE10" s="27" t="str">
-        <x:v>半导体车间；文中含480任务锚点与灵敏度分析</x:v>
+        <x:v>半导体车间小规模与480任务大规模仿真</x:v>
       </x:c>
       <x:c r="AF10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>运输任务；大规模480任务</x:v>
       </x:c>
       <x:c r="AG10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>半导体工位，数量见算例</x:v>
       </x:c>
       <x:c r="AI10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>多AGV，数量见算例</x:v>
       </x:c>
       <x:c r="AJ10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>半导体有向路网</x:v>
       </x:c>
       <x:c r="AK10" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>小/大规模</x:v>
       </x:c>
       <x:c r="AL10" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>两阶段方法与分配/路径规则对照</x:v>
       </x:c>
       <x:c r="AM10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>停止为任务完成；计算预算未报告</x:v>
       </x:c>
       <x:c r="AN10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>停止为任务完成；计算预算未报告</x:v>
       </x:c>
       <x:c r="AO10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ10" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR10" s="27" t="str">
-        <x:v>效率；安全</x:v>
+        <x:v>完成时间、运输/等待、冲突及灵敏度</x:v>
       </x:c>
       <x:c r="AS10" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3618,13 +3618,13 @@
         <x:v>直接：摘要/关键词；“两阶段算法”；“碰撞检测与避免”；“480”；半导体车间；文中含480任务锚点与灵敏度分析</x:v>
       </x:c>
       <x:c r="AV10" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B007 `2.2`、`3 AGV碰撞检测及避免算法`；B007 `4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="AW10" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX10" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY10" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3633,7 +3633,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA10" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB10" s="27" t="str">
         <x:v>OK</x:v>
@@ -3647,7 +3647,7 @@
         <x:v>L008</x:v>
       </x:c>
       <x:c r="C11" s="27" t="str">
-        <x:v>B008；直接：摘要“碰撞问题和死锁问题”“启发式算法和强化学习算法”</x:v>
+        <x:v>B008 第2章、`3 结论与展望`；B008 第2章</x:v>
       </x:c>
       <x:c r="D11" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -3713,64 +3713,64 @@
         <x:v>综述；原分类=跨类型（综述）；跨/跨</x:v>
       </x:c>
       <x:c r="Y11" s="27" t="str">
-        <x:v>综述：仓库多AGV碰撞/死锁、启发式与强化学习方法</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="Z11" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AA11" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>按碰撞、死锁及启发式/强化学习方法归纳</x:v>
       </x:c>
       <x:c r="AB11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AC11" s="27" t="str">
-        <x:v>综述：仓库多AGV碰撞/死锁、启发式与强化学习方法</x:v>
+        <x:v>方法分类与趋势综合，不构成单一调用链</x:v>
       </x:c>
       <x:c r="AD11" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>方法分类与趋势综合，不构成单一调用链</x:v>
       </x:c>
       <x:c r="AE11" s="27" t="str">
-        <x:v>综述，无统一实验协议</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AF11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AG11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AH11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AI11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AJ11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>仓储路网综述</x:v>
       </x:c>
       <x:c r="AK11" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>综述</x:v>
       </x:c>
       <x:c r="AL11" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AM11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AN11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AO11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AP11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AQ11" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AR11" s="27" t="str">
-        <x:v>安全；效率；跨类型（综述）</x:v>
+        <x:v>无统一实验指标</x:v>
       </x:c>
       <x:c r="AS11" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3782,13 +3782,13 @@
         <x:v>直接：摘要“碰撞问题和死锁问题”“启发式算法和强化学习算法”；综述，无统一实验协议</x:v>
       </x:c>
       <x:c r="AV11" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B008 第2章、`3 结论与展望`；B008 第2章</x:v>
       </x:c>
       <x:c r="AW11" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX11" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6字段已完成原文深度抽取</x:v>
       </x:c>
       <x:c r="AY11" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3797,7 +3797,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA11" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB11" s="27" t="str">
         <x:v>OK</x:v>
@@ -3811,7 +3811,7 @@
         <x:v>L009</x:v>
       </x:c>
       <x:c r="C12" s="27" t="str">
-        <x:v>B009；直接：关键词；“集中式调度和分布式调度”；任务分配；路径规划；展望</x:v>
+        <x:v>B009 第2–3章及展望；B009 第2–3章</x:v>
       </x:c>
       <x:c r="D12" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -3877,64 +3877,64 @@
         <x:v>综述；原分类=跨类型（综述）；跨/跨</x:v>
       </x:c>
       <x:c r="Y12" s="27" t="str">
-        <x:v>综述：集中式/分布式任务分配、路径规划与协商</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="Z12" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AA12" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>归纳集中/分布式任务分配、路径协商与冲突协调</x:v>
       </x:c>
       <x:c r="AB12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AC12" s="27" t="str">
-        <x:v>综述：集中式/分布式任务分配、路径规划与协商</x:v>
+        <x:v>任务分配→路径规划→通信/协商的综述链</x:v>
       </x:c>
       <x:c r="AD12" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>任务分配→路径规划→通信/协商的综述链</x:v>
       </x:c>
       <x:c r="AE12" s="27" t="str">
-        <x:v>综述，无统一实验协议</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AF12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AG12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AH12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AI12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AJ12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>跨场景综述</x:v>
       </x:c>
       <x:c r="AK12" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>综述</x:v>
       </x:c>
       <x:c r="AL12" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AM12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AN12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AO12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AP12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AQ12" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用（综述）</x:v>
       </x:c>
       <x:c r="AR12" s="27" t="str">
-        <x:v>效率；鲁棒性；跨类型（综述）</x:v>
+        <x:v>无统一实验指标</x:v>
       </x:c>
       <x:c r="AS12" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -3946,13 +3946,13 @@
         <x:v>直接：关键词；“集中式调度和分布式调度”；任务分配；路径规划；展望；综述，无统一实验协议</x:v>
       </x:c>
       <x:c r="AV12" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B009 第2–3章及展望；B009 第2–3章</x:v>
       </x:c>
       <x:c r="AW12" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX12" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6字段已完成原文深度抽取</x:v>
       </x:c>
       <x:c r="AY12" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -3961,7 +3961,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA12" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB12" s="27" t="str">
         <x:v>OK</x:v>
@@ -3975,7 +3975,7 @@
         <x:v>L010</x:v>
       </x:c>
       <x:c r="C13" s="27" t="str">
-        <x:v>B010；直接：摘要；`DMA-DDQN`；多智能体；联合调度；奖励成形</x:v>
+        <x:v>B010 强化学习环境、`2.5 训练及参数调优`；B010 `2.5`、`3 数值实验`</x:v>
       </x:c>
       <x:c r="D13" s="27" t="str">
         <x:v>Verified</x:v>
@@ -4041,64 +4041,64 @@
         <x:v>核心车间原始研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y13" s="27" t="str">
-        <x:v>DMA-DDQN多智能体强化学习＋奖励成形</x:v>
+        <x:v>工件、机器、AGV局部状态；多智能体联合动作</x:v>
       </x:c>
       <x:c r="Z13" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>规则动作执行后推进加工/运输环境并形成分步与终局奖励</x:v>
       </x:c>
       <x:c r="AA13" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>可行规则限定动作，不另报染色体修复</x:v>
       </x:c>
       <x:c r="AB13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>完成调度回合；训练停止按原文参数</x:v>
       </x:c>
       <x:c r="AC13" s="27" t="str">
-        <x:v>DMA-DDQN多智能体强化学习＋奖励成形</x:v>
+        <x:v>DMA-DDQN：智能体观测→联合选规则→环境更新→经验回放/目标网络更新；奖励成形嵌入训练</x:v>
       </x:c>
       <x:c r="AD13" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>DMA-DDQN：智能体观测→联合选规则→环境更新→经验回放/目标网络更新；奖励成形嵌入训练</x:v>
       </x:c>
       <x:c r="AE13" s="27" t="str">
-        <x:v>不同规模与规则/GA/DQN对比；重复和统计待N6抽取</x:v>
+        <x:v>不同规模FJSP联合调度算例</x:v>
       </x:c>
       <x:c r="AF13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见数值实验</x:v>
       </x:c>
       <x:c r="AG13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见数值实验</x:v>
       </x:c>
       <x:c r="AH13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见数值实验</x:v>
       </x:c>
       <x:c r="AI13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见数值实验</x:v>
       </x:c>
       <x:c r="AJ13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>车间联合调度环境</x:v>
       </x:c>
       <x:c r="AK13" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多规模</x:v>
       </x:c>
       <x:c r="AL13" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>调度规则、GA、DQN及DMA-DDQN消融/变体</x:v>
       </x:c>
       <x:c r="AM13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练及调参见§2.5；完整统一预算未报告</x:v>
       </x:c>
       <x:c r="AN13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练及调参见§2.5；完整统一预算未报告</x:v>
       </x:c>
       <x:c r="AO13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ13" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR13" s="27" t="str">
-        <x:v>效率；多目标组合</x:v>
+        <x:v>makespan及文内多目标/奖励表现</x:v>
       </x:c>
       <x:c r="AS13" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4110,13 +4110,13 @@
         <x:v>直接：摘要；`DMA-DDQN`；多智能体；联合调度；奖励成形；不同规模与规则/GA/DQN对比；重复和统计待N6抽取</x:v>
       </x:c>
       <x:c r="AV13" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B010 强化学习环境、`2.5 训练及参数调优`；B010 `2.5`、`3 数值实验`</x:v>
       </x:c>
       <x:c r="AW13" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX13" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY13" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4125,7 +4125,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA13" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB13" s="27" t="str">
         <x:v>OK</x:v>
@@ -4139,7 +4139,7 @@
         <x:v>L011</x:v>
       </x:c>
       <x:c r="C14" s="27" t="str">
-        <x:v>B011；直接：题名/关键词；数学模型；编码；FT06/FT10；Conclusion</x:v>
+        <x:v>B011 `2.3`–`2.5`、图7；B011 表2–3、`4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="D14" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -4205,64 +4205,64 @@
         <x:v>核心车间原始研究；原分类=元启发式；静/确</x:v>
       </x:c>
       <x:c r="Y14" s="27" t="str">
-        <x:v>改进花授粉算法IFPA＋CSM/PCA机制</x:v>
+        <x:v>基于工序的整数序列</x:v>
       </x:c>
       <x:c r="Z14" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>依次确定工序机器、加工时段与 AGV配送时段</x:v>
       </x:c>
       <x:c r="AA14" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>连续 FPA 新解按旧序列键值排序修复为合法工序序列</x:v>
       </x:c>
       <x:c r="AB14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>150 代</x:v>
       </x:c>
       <x:c r="AC14" s="27" t="str">
-        <x:v>改进花授粉算法IFPA＋CSM/PCA机制</x:v>
+        <x:v>改进初始化→FPA全局/局部授粉→PCA启发式变异→SA概率接受；GA交叉嵌入FPA</x:v>
       </x:c>
       <x:c r="AD14" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>改进初始化→FPA全局/局部授粉→PCA启发式变异→SA概率接受；GA交叉嵌入FPA</x:v>
       </x:c>
       <x:c r="AE14" s="27" t="str">
-        <x:v>FT06、FT10与平台实验；精度/稳定性文内比较</x:v>
+        <x:v>FT06、FT10、LA01–LA08；单/多AGV原型实验</x:v>
       </x:c>
       <x:c r="AF14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>FT06/FT10/LA01–08及原型任务</x:v>
       </x:c>
       <x:c r="AG14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>随标准JSP实例</x:v>
       </x:c>
       <x:c r="AH14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>随标准JSP实例</x:v>
       </x:c>
       <x:c r="AI14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>单/多AGV原型</x:v>
       </x:c>
       <x:c r="AJ14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>实验原型布局</x:v>
       </x:c>
       <x:c r="AK14" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>标准实例+原型</x:v>
       </x:c>
       <x:c r="AL14" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>FPA、GA及集成调度对照</x:v>
       </x:c>
       <x:c r="AM14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=60，150代；T0=800、q=.92等</x:v>
       </x:c>
       <x:c r="AN14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>pop=60，150代；T0=800、q=.92等</x:v>
       </x:c>
       <x:c r="AO14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="AP14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ14" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR14" s="27" t="str">
-        <x:v>效率；稳定性</x:v>
+        <x:v>min、max、mean、makespan、AGV利用率</x:v>
       </x:c>
       <x:c r="AS14" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4274,13 +4274,13 @@
         <x:v>直接：题名/关键词；数学模型；编码；FT06/FT10；Conclusion；FT06、FT10与平台实验；精度/稳定性文内比较</x:v>
       </x:c>
       <x:c r="AV14" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B011 `2.3`–`2.5`、图7；B011 表2–3、`4.1`–`4.2`</x:v>
       </x:c>
       <x:c r="AW14" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX14" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY14" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4289,7 +4289,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA14" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB14" s="27" t="str">
         <x:v>OK</x:v>
@@ -4303,7 +4303,7 @@
         <x:v>L012</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>B012；直接：摘要；“多步长动作”“动态奖励”；单车路径与多任务实验；随机性未见报告</x:v>
+        <x:v>B012 `2 改进PPO算法`、`2.4 算法流程`；B012 第4章</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>Verified</x:v>
@@ -4369,64 +4369,64 @@
         <x:v>路径/任务相邻研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y15" s="27" t="str">
-        <x:v>改进PPO＋多步长动作＋动态奖励</x:v>
+        <x:v>栅格状态、位置/目标/障碍及多步长离散动作</x:v>
       </x:c>
       <x:c r="Z15" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>PPO 动作推进 AGV 并返回距离/碰撞奖励</x:v>
       </x:c>
       <x:c r="AA15" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>越界和碰撞惩罚；动态奖励抑制无效动作</x:v>
       </x:c>
       <x:c r="AB15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>达到目标或回合上限；训练轮次见实验</x:v>
       </x:c>
       <x:c r="AC15" s="27" t="str">
-        <x:v>改进PPO＋多步长动作＋动态奖励</x:v>
+        <x:v>PPO采样→优势估计→裁剪目标更新；多步长动作与动态奖励嵌入动作/奖励层</x:v>
       </x:c>
       <x:c r="AD15" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>PPO采样→优势估计→裁剪目标更新；多步长动作与动态奖励嵌入动作/奖励层</x:v>
       </x:c>
       <x:c r="AE15" s="27" t="str">
-        <x:v>单车路径与多任务实验；距离和收敛效率</x:v>
+        <x:v>单AGV路径与多任务调度仿真地图</x:v>
       </x:c>
       <x:c r="AF15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>单车路径与多任务</x:v>
       </x:c>
       <x:c r="AG15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>单AGV</x:v>
       </x:c>
       <x:c r="AJ15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>栅格地图</x:v>
       </x:c>
       <x:c r="AK15" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>单车/多任务</x:v>
       </x:c>
       <x:c r="AL15" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>PPO及传统路径/任务方法</x:v>
       </x:c>
       <x:c r="AM15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>超参数见原文；达到目标或回合上限</x:v>
       </x:c>
       <x:c r="AN15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>超参数见原文；达到目标或回合上限</x:v>
       </x:c>
       <x:c r="AO15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ15" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR15" s="27" t="str">
-        <x:v>效率；计算成本</x:v>
+        <x:v>路径长度、训练收敛、任务总距离/效率</x:v>
       </x:c>
       <x:c r="AS15" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4438,13 +4438,13 @@
         <x:v>直接：摘要；“多步长动作”“动态奖励”；单车路径与多任务实验；随机性未见报告；单车路径与多任务实验；距离和收敛效率</x:v>
       </x:c>
       <x:c r="AV15" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B012 `2 改进PPO算法`、`2.4 算法流程`；B012 第4章</x:v>
       </x:c>
       <x:c r="AW15" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX15" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY15" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4453,7 +4453,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA15" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB15" s="27" t="str">
         <x:v>OK</x:v>
@@ -4467,7 +4467,7 @@
         <x:v>L013</x:v>
       </x:c>
       <x:c r="C16" s="27" t="str">
-        <x:v>B013；直接：摘要“网格地图”“防冲突路径规划”“最大完工时间”</x:v>
+        <x:v>B013 `2.2.5 算法步骤`、式(34)、`3.1`；B013 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="D16" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -4533,64 +4533,64 @@
         <x:v>路径/任务相邻研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y16" s="27" t="str">
-        <x:v>改进PPO防绕远与防冲突路径规划</x:v>
+        <x:v>码头栅格、各AGV位置/目标及联合路径状态</x:v>
       </x:c>
       <x:c r="Z16" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>PPO逐步选择下一节点</x:v>
       </x:c>
       <x:c r="AA16" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>节点/相向冲突、越界强惩罚；防绕远奖励项</x:v>
       </x:c>
       <x:c r="AB16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>到达目标/非法终止；训练300轮</x:v>
       </x:c>
       <x:c r="AC16" s="27" t="str">
-        <x:v>改进PPO防绕远与防冲突路径规划</x:v>
+        <x:v>PPO采样更新；防绕远机制嵌入奖励函数</x:v>
       </x:c>
       <x:c r="AD16" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>PPO采样更新；防绕远机制嵌入奖励函数</x:v>
       </x:c>
       <x:c r="AE16" s="27" t="str">
-        <x:v>码头网格与规模实验；求解速度和路径指标</x:v>
+        <x:v>11×11、21×21、31×31双向路网；AGV数3–30</x:v>
       </x:c>
       <x:c r="AF16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>码头运输任务</x:v>
       </x:c>
       <x:c r="AG16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>岸桥/堆场节点</x:v>
       </x:c>
       <x:c r="AI16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>3/5/10；5/10/15；20/25/30</x:v>
       </x:c>
       <x:c r="AJ16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>11×11、21×21、31×31双向车道</x:v>
       </x:c>
       <x:c r="AK16" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>小/中/大</x:v>
       </x:c>
       <x:c r="AL16" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>标准PPO/去防绕远机制及参数对照</x:v>
       </x:c>
       <x:c r="AM16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练300轮</x:v>
       </x:c>
       <x:c r="AN16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练300轮</x:v>
       </x:c>
       <x:c r="AO16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ16" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>报告参数差异p值；检验名称以原文为准</x:v>
       </x:c>
       <x:c r="AR16" s="27" t="str">
-        <x:v>效率；稳定性；安全</x:v>
+        <x:v>累积奖励、步数、路径长度、冲突/成功</x:v>
       </x:c>
       <x:c r="AS16" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4602,13 +4602,13 @@
         <x:v>直接：摘要“网格地图”“防冲突路径规划”“最大完工时间”；码头网格与规模实验；求解速度和路径指标</x:v>
       </x:c>
       <x:c r="AV16" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B013 `2.2.5 算法步骤`、式(34)、`3.1`；B013 `3.1`–`3.3`</x:v>
       </x:c>
       <x:c r="AW16" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX16" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY16" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4617,7 +4617,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA16" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB16" s="27" t="str">
         <x:v>OK</x:v>
@@ -4631,7 +4631,7 @@
         <x:v>L014</x:v>
       </x:c>
       <x:c r="C17" s="27" t="str">
-        <x:v>B014；直接：摘要；YOLOv8；PPO-LSTM；“个人空间”；限制：行人运动随机模型当前不清楚</x:v>
+        <x:v>B014 系统架构、`2.3 LSTM-PPO`、奖惩机制；B014 `4.2`、第5章</x:v>
       </x:c>
       <x:c r="D17" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -4697,64 +4697,64 @@
         <x:v>路径/任务相邻研究；原分类=学习型；动/不清楚</x:v>
       </x:c>
       <x:c r="Y17" s="27" t="str">
-        <x:v>YOLOv8感知＋PPO-LSTM避让控制</x:v>
+        <x:v>RGB/深度图、AGV位姿、目标与YOLOv8行人状态</x:v>
       </x:c>
       <x:c r="Z17" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>LSTM-PPO输出连续运动动作，Isaac Sim推进</x:v>
       </x:c>
       <x:c r="AA17" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>碰撞/越界终止；个人空间分层惩罚</x:v>
       </x:c>
       <x:c r="AB17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>到达目标、碰撞/越界或回合上限</x:v>
       </x:c>
       <x:c r="AC17" s="27" t="str">
-        <x:v>YOLOv8感知＋PPO-LSTM避让控制</x:v>
+        <x:v>YOLOv8特征→CNN/LSTM策略与价值网络→PPO更新；先无行人预训练再正式训练</x:v>
       </x:c>
       <x:c r="AD17" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>YOLOv8特征→CNN/LSTM策略与价值网络→PPO更新；先无行人预训练再正式训练</x:v>
       </x:c>
       <x:c r="AE17" s="27" t="str">
-        <x:v>仿真实验；安全距离与效率指标</x:v>
+        <x:v>Isaac Sim虚拟工厂；单AGV–行人；30轮测试</x:v>
       </x:c>
       <x:c r="AF17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>单AGV行人避让任务</x:v>
       </x:c>
       <x:c r="AG17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AJ17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>Isaac Sim虚拟工厂</x:v>
       </x:c>
       <x:c r="AK17" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>单AGV案例</x:v>
       </x:c>
       <x:c r="AL17" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>PPO（无LSTM）</x:v>
       </x:c>
       <x:c r="AM17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>预训练6×10^5步；正式训练约2.3×10^5步收敛</x:v>
       </x:c>
       <x:c r="AN17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>预训练6×10^5步；正式训练约2.3×10^5步收敛</x:v>
       </x:c>
       <x:c r="AO17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="AP17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ17" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR17" s="27" t="str">
-        <x:v>安全；效率</x:v>
+        <x:v>平均回合奖励、避障成功率、舒适成功率、最小距离</x:v>
       </x:c>
       <x:c r="AS17" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4766,13 +4766,13 @@
         <x:v>直接：摘要；YOLOv8；PPO-LSTM；“个人空间”；限制：行人运动随机模型当前不清楚；仿真实验；安全距离与效率指标</x:v>
       </x:c>
       <x:c r="AV17" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B014 系统架构、`2.3 LSTM-PPO`、奖惩机制；B014 `4.2`、第5章</x:v>
       </x:c>
       <x:c r="AW17" s="27" t="str">
         <x:v>随机性/事件生成机制不完整</x:v>
       </x:c>
       <x:c r="AX17" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY17" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4781,7 +4781,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA17" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB17" s="27" t="str">
         <x:v>OK</x:v>
@@ -4795,7 +4795,7 @@
         <x:v>L015</x:v>
       </x:c>
       <x:c r="C18" s="27" t="str">
-        <x:v>B015；直接：摘要“工件智能体”“小车智能体”“交互”“小车位置”</x:v>
+        <x:v>B015 `2.2 调度流程`、`2.3 学习过程`；B015 案例段与图6</x:v>
       </x:c>
       <x:c r="D18" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -4861,64 +4861,64 @@
         <x:v>核心车间原始研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y18" s="27" t="str">
-        <x:v>工件智能体DQN＋AGV智能体DQN交互调度</x:v>
+        <x:v>工件/机器/小车状态；两个智能体输出规则权重</x:v>
       </x:c>
       <x:c r="Z18" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>工件智能体先定工件/机器，小车智能体接收其决策后定AGV并推进</x:v>
       </x:c>
       <x:c r="AA18" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>动作由可执行规则集合限制</x:v>
       </x:c>
       <x:c r="AB18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>完成全部工件</x:v>
       </x:c>
       <x:c r="AC18" s="27" t="str">
-        <x:v>工件智能体DQN＋AGV智能体DQN交互调度</x:v>
+        <x:v>两智能体依次观测→ε-greedy选权重动作→环境执行→DQN经验学习</x:v>
       </x:c>
       <x:c r="AD18" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>两智能体依次观测→ε-greedy选权重动作→环境执行→DQN经验学习</x:v>
       </x:c>
       <x:c r="AE18" s="27" t="str">
-        <x:v>离散制造案例；综合调度与负载指标</x:v>
+        <x:v>实际案例：4工件、9机器、3AGV、16次搬运</x:v>
       </x:c>
       <x:c r="AF18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>工序数不等</x:v>
       </x:c>
       <x:c r="AH18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="AI18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AJ18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>实际离散制造车间布局</x:v>
       </x:c>
       <x:c r="AK18" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>案例</x:v>
       </x:c>
       <x:c r="AL18" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>文献[21]算法</x:v>
       </x:c>
       <x:c r="AM18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>全部工件完成；训练预算未报告</x:v>
       </x:c>
       <x:c r="AN18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>全部工件完成；训练预算未报告</x:v>
       </x:c>
       <x:c r="AO18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ18" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR18" s="27" t="str">
-        <x:v>效率；负载均衡；多目标组合</x:v>
+        <x:v>makespan、AGV搬运次数均衡</x:v>
       </x:c>
       <x:c r="AS18" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -4930,13 +4930,13 @@
         <x:v>直接：摘要“工件智能体”“小车智能体”“交互”“小车位置”；离散制造案例；综合调度与负载指标</x:v>
       </x:c>
       <x:c r="AV18" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B015 `2.2 调度流程`、`2.3 学习过程`；B015 案例段与图6</x:v>
       </x:c>
       <x:c r="AW18" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX18" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY18" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -4945,7 +4945,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA18" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB18" s="27" t="str">
         <x:v>OK</x:v>
@@ -4959,7 +4959,7 @@
         <x:v>L016</x:v>
       </x:c>
       <x:c r="C19" s="27" t="str">
-        <x:v>B016；直接：摘要“工件动态到达”“工时不确定”“右移/完全重调度”“时间窗”；限制：转换文本存在缺字</x:v>
+        <x:v>B016 `2.1 算法框架`、时间窗A*、组合重调度；B016 表4、动态试验</x:v>
       </x:c>
       <x:c r="D19" s="27" t="str">
         <x:v>Verified</x:v>
@@ -5025,64 +5025,64 @@
         <x:v>核心车间原始研究；原分类=混合；动/随</x:v>
       </x:c>
       <x:c r="Y19" s="27" t="str">
-        <x:v>右移/完全重调度＋时间窗路径机制；部分算法字符串待原PDF复核</x:v>
+        <x:v>工件、机器、AGV与时窗路径状态；9个复合规则动作</x:v>
       </x:c>
       <x:c r="Z19" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>规则组合决定工件/机器/AGV，时窗A*生成无冲突路径</x:v>
       </x:c>
       <x:c r="AA19" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>工时延误先判干涉；右移与完全重调度择优</x:v>
       </x:c>
       <x:c r="AB19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最后工序结束；动态仿真时钟结束</x:v>
       </x:c>
       <x:c r="AC19" s="27" t="str">
-        <x:v>右移/完全重调度＋时间窗路径机制；部分算法字符串待原PDF复核</x:v>
+        <x:v>DQN选择复合规则；事件+周期触发组合重调度，评价相同时优先右移</x:v>
       </x:c>
       <x:c r="AD19" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>DQN选择复合规则；事件+周期触发组合重调度，评价相同时优先右移</x:v>
       </x:c>
       <x:c r="AE19" s="27" t="str">
-        <x:v>动态到达/工时不确定案例；转换缺字限制</x:v>
+        <x:v>4/4、4/6、7/6、10/8工件/机器；AGV 2–7；另有动态到达与随机工时案例</x:v>
       </x:c>
       <x:c r="AF19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>4/4、4/6、7/6、10/8中的工件数</x:v>
       </x:c>
       <x:c r="AG19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见案例</x:v>
       </x:c>
       <x:c r="AH19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>4/6/6/8</x:v>
       </x:c>
       <x:c r="AI19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>2–7</x:v>
       </x:c>
       <x:c r="AJ19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>拓扑地图+时间窗</x:v>
       </x:c>
       <x:c r="AK19" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>四档案例+动态案例</x:v>
       </x:c>
       <x:c r="AL19" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>文献算法；右移与完全重调度</x:v>
       </x:c>
       <x:c r="AM19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最后工序结束；网络训练预算未完整报告</x:v>
       </x:c>
       <x:c r="AN19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最后工序结束；网络训练预算未完整报告</x:v>
       </x:c>
       <x:c r="AO19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ19" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR19" s="27" t="str">
-        <x:v>效率；稳定性；多目标组合</x:v>
+        <x:v>makespan、总拖期、机器利用率、Td/Dd/Y</x:v>
       </x:c>
       <x:c r="AS19" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5094,13 +5094,13 @@
         <x:v>直接：摘要“工件动态到达”“工时不确定”“右移/完全重调度”“时间窗”；限制：转换文本存在缺字；动态到达/工时不确定案例；转换缺字限制</x:v>
       </x:c>
       <x:c r="AV19" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B016 `2.1 算法框架`、时间窗A*、组合重调度；B016 表4、动态试验</x:v>
       </x:c>
       <x:c r="AW19" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX19" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY19" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5109,7 +5109,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA19" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB19" s="27" t="str">
         <x:v>OK</x:v>
@@ -5123,7 +5123,7 @@
         <x:v>L017</x:v>
       </x:c>
       <x:c r="C20" s="27" t="str">
-        <x:v>B017；直接：题名/摘要；“变速充电AGV”；MSPPO；析取图；HV/IGD</x:v>
+        <x:v>B017 `2 MSPPO算法`、`2.4 算法框架`；B017 `3.1`、`3.4`</x:v>
       </x:c>
       <x:c r="D20" s="27" t="str">
         <x:v>Verified</x:v>
@@ -5189,64 +5189,64 @@
         <x:v>核心车间原始研究；原分类=学习型；静/确</x:v>
       </x:c>
       <x:c r="Y20" s="27" t="str">
-        <x:v>MSPPO＋析取图；变速与充电联合决策</x:v>
+        <x:v>工序、机器、AGV、速度/充电状态的析取图表示</x:v>
       </x:c>
       <x:c r="Z20" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>策略动作后更新加工、运输、电量和充电</x:v>
       </x:c>
       <x:c r="AA20" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>可行规则与析取图约束排除冲突</x:v>
       </x:c>
       <x:c r="AB20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>完成所有工序/训练回合</x:v>
       </x:c>
       <x:c r="AC20" s="27" t="str">
-        <x:v>MSPPO＋析取图；变速与充电联合决策</x:v>
+        <x:v>多策略PPO在联合调度环境中选复合动作；多策略网络嵌入PPO</x:v>
       </x:c>
       <x:c r="AD20" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>多策略PPO在联合调度环境中选复合动作；多策略网络嵌入PPO</x:v>
       </x:c>
       <x:c r="AE20" s="27" t="str">
-        <x:v>多目标算例；HV/IGD；完整参考点和重复待N6抽取</x:v>
+        <x:v>绿色FJSP与变速充电AGV算例</x:v>
       </x:c>
       <x:c r="AF20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验算例</x:v>
       </x:c>
       <x:c r="AG20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验算例</x:v>
       </x:c>
       <x:c r="AH20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验算例</x:v>
       </x:c>
       <x:c r="AI20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验算例</x:v>
       </x:c>
       <x:c r="AJ20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>车间运输/充电布局</x:v>
       </x:c>
       <x:c r="AK20" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多规模</x:v>
       </x:c>
       <x:c r="AL20" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>NSGA-II及文内多目标算法</x:v>
       </x:c>
       <x:c r="AM20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§3.1；完整预算按原文表</x:v>
       </x:c>
       <x:c r="AN20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§3.1；完整预算按原文表</x:v>
       </x:c>
       <x:c r="AO20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ20" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR20" s="27" t="str">
-        <x:v>效率；能源；多目标组合</x:v>
+        <x:v>makespan、能耗、HV、IGD</x:v>
       </x:c>
       <x:c r="AS20" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5258,13 +5258,13 @@
         <x:v>直接：题名/摘要；“变速充电AGV”；MSPPO；析取图；HV/IGD；多目标算例；HV/IGD；完整参考点和重复待N6抽取</x:v>
       </x:c>
       <x:c r="AV20" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B017 `2 MSPPO算法`、`2.4 算法框架`；B017 `3.1`、`3.4`</x:v>
       </x:c>
       <x:c r="AW20" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX20" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY20" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5273,7 +5273,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA20" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB20" s="27" t="str">
         <x:v>OK</x:v>
@@ -5287,7 +5287,7 @@
         <x:v>L018</x:v>
       </x:c>
       <x:c r="C21" s="27" t="str">
-        <x:v>B018；直接：摘要“完工时间、AGV数量、惩罚成本”“多段式实数编码”</x:v>
+        <x:v>B018 `2.1 算法流程`、`2.2 编码设计`；B018 `3 算例`</x:v>
       </x:c>
       <x:c r="D21" s="27" t="str">
         <x:v>Verified</x:v>
@@ -5353,64 +5353,64 @@
         <x:v>核心车间原始研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y21" s="27" t="str">
-        <x:v>AMOGA-DE＋多段式实数编码</x:v>
+        <x:v>多AGV调度染色体</x:v>
       </x:c>
       <x:c r="Z21" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>按染色体生成任务顺序与车辆计划</x:v>
       </x:c>
       <x:c r="AA21" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>变异/差分更新后进行可行性处理</x:v>
       </x:c>
       <x:c r="AB21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>达到最大迭代</x:v>
       </x:c>
       <x:c r="AC21" s="27" t="str">
-        <x:v>AMOGA-DE＋多段式实数编码</x:v>
+        <x:v>AMOGA 主循环中嵌入差分进化与外部精英/非支配选择</x:v>
       </x:c>
       <x:c r="AD21" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>AMOGA 主循环中嵌入差分进化与外部精英/非支配选择</x:v>
       </x:c>
       <x:c r="AE21" s="27" t="str">
-        <x:v>3个规模；NSGA-II/SPEA2对比</x:v>
+        <x:v>3种规模多AGV车间算例</x:v>
       </x:c>
       <x:c r="AF21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见三种规模算例</x:v>
       </x:c>
       <x:c r="AG21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>多AGV</x:v>
       </x:c>
       <x:c r="AJ21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>智能车间布局</x:v>
       </x:c>
       <x:c r="AK21" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>三档</x:v>
       </x:c>
       <x:c r="AL21" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>NSGA-II、SPEA2</x:v>
       </x:c>
       <x:c r="AM21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数与迭代见§3</x:v>
       </x:c>
       <x:c r="AN21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数与迭代见§3</x:v>
       </x:c>
       <x:c r="AO21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ21" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR21" s="27" t="str">
-        <x:v>效率；资源成本；多目标组合</x:v>
+        <x:v>多目标值、Pareto分布、收敛/多样性</x:v>
       </x:c>
       <x:c r="AS21" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5422,13 +5422,13 @@
         <x:v>直接：摘要“完工时间、AGV数量、惩罚成本”“多段式实数编码”；3个规模；NSGA-II/SPEA2对比</x:v>
       </x:c>
       <x:c r="AV21" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B018 `2.1 算法流程`、`2.2 编码设计`；B018 `3 算例`</x:v>
       </x:c>
       <x:c r="AW21" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX21" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY21" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5437,7 +5437,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA21" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB21" s="27" t="str">
         <x:v>OK</x:v>
@@ -5451,7 +5451,7 @@
         <x:v>L019</x:v>
       </x:c>
       <x:c r="C22" s="27" t="str">
-        <x:v>B019；直接：摘要/模型；GAIVNS；三层编码；关键路径；配置实验</x:v>
+        <x:v>B019 `2.2.1 编码和解码`、GAIVNS流程；B019 `3.1`–`4.2`</x:v>
       </x:c>
       <x:c r="D22" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -5517,64 +5517,64 @@
         <x:v>核心车间原始研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y22" s="27" t="str">
-        <x:v>GAIVNS＋三层编码＋关键路径局部搜索</x:v>
+        <x:v>OS–MS–AS 三层编码</x:v>
       </x:c>
       <x:c r="Z22" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>顺序解码机器加工与AGV运输</x:v>
       </x:c>
       <x:c r="AA22" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>邻域后保持工序次数、机器资格与车辆编号合法</x:v>
       </x:c>
       <x:c r="AB22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>达到最大迭代</x:v>
       </x:c>
       <x:c r="AC22" s="27" t="str">
-        <x:v>GAIVNS＋三层编码＋关键路径局部搜索</x:v>
+        <x:v>GA全局进化后在关键路径上执行改进VNS；局部搜索为代内改进插入点</x:v>
       </x:c>
       <x:c r="AD22" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>GA全局进化后在关键路径上执行改进VNS；局部搜索为代内改进插入点</x:v>
       </x:c>
       <x:c r="AE22" s="27" t="str">
-        <x:v>标准算例＋企业案例＋配置/敏感性实验</x:v>
+        <x:v>标准算例、企业案例与12/96组配置试验</x:v>
       </x:c>
       <x:c r="AF22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>标准算例与企业案例</x:v>
       </x:c>
       <x:c r="AG22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AH22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AI22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见配置实验</x:v>
       </x:c>
       <x:c r="AJ22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>车间运输矩阵</x:v>
       </x:c>
       <x:c r="AK22" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>标准+企业案例</x:v>
       </x:c>
       <x:c r="AL22" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>GA及文内先进算法</x:v>
       </x:c>
       <x:c r="AM22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§3.1；最大迭代停止</x:v>
       </x:c>
       <x:c r="AN22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§3.1；最大迭代停止</x:v>
       </x:c>
       <x:c r="AO22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ22" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR22" s="27" t="str">
-        <x:v>效率；多目标组合</x:v>
+        <x:v>makespan、AGV配置边际、相对差距/求解时间</x:v>
       </x:c>
       <x:c r="AS22" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5586,13 +5586,13 @@
         <x:v>直接：摘要/模型；GAIVNS；三层编码；关键路径；配置实验；标准算例＋企业案例＋配置/敏感性实验</x:v>
       </x:c>
       <x:c r="AV22" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B019 `2.2.1 编码和解码`、GAIVNS流程；B019 `3.1`–`4.2`</x:v>
       </x:c>
       <x:c r="AW22" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX22" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY22" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5601,7 +5601,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA22" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB22" s="27" t="str">
         <x:v>OK</x:v>
@@ -5615,7 +5615,7 @@
         <x:v>L020</x:v>
       </x:c>
       <x:c r="C23" s="27" t="str">
-        <x:v>B020；直接：摘要“高峰和低谷时段”“充电策略”“能量均衡”；限制：任务场景给定，未见概率事件模型</x:v>
+        <x:v>B020 `2.1 算法设计`、`3.1 仿真实验`；B020 `3.1 仿真实验`</x:v>
       </x:c>
       <x:c r="D23" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -5681,64 +5681,64 @@
         <x:v>路径/任务相邻研究；原分类=混合；动/确</x:v>
       </x:c>
       <x:c r="Y23" s="27" t="str">
-        <x:v>MADDPG-PGT势博弈深度强化学习＋充电策略</x:v>
+        <x:v>多AGV局部观测、连续动作与电量状态</x:v>
       </x:c>
       <x:c r="Z23" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>MADDPG执行联合动作并推进码头运输环境</x:v>
       </x:c>
       <x:c r="AA23" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>势博弈奖励/约束协调能量均衡与冲突</x:v>
       </x:c>
       <x:c r="AB23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练回合/任务完成</x:v>
       </x:c>
       <x:c r="AC23" s="27" t="str">
-        <x:v>MADDPG-PGT势博弈深度强化学习＋充电策略</x:v>
+        <x:v>集中训练分散执行；势博弈项嵌入MADDPG奖励与策略更新</x:v>
       </x:c>
       <x:c r="AD23" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>集中训练分散执行；势博弈项嵌入MADDPG奖励与策略更新</x:v>
       </x:c>
       <x:c r="AE23" s="27" t="str">
-        <x:v>3艘实际船舶场景；能量均衡与效率指标</x:v>
+        <x:v>3艘实际船舶数据的码头AGV群仿真</x:v>
       </x:c>
       <x:c r="AF23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>3艘实际船舶任务</x:v>
       </x:c>
       <x:c r="AG23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>码头作业资源</x:v>
       </x:c>
       <x:c r="AI23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>AGV群，数量见实验</x:v>
       </x:c>
       <x:c r="AJ23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>自动化码头</x:v>
       </x:c>
       <x:c r="AK23" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>实际数据案例</x:v>
       </x:c>
       <x:c r="AL23" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>MADDPG等DRL/无势博弈对照</x:v>
       </x:c>
       <x:c r="AM23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练参数见§3.1</x:v>
       </x:c>
       <x:c r="AN23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练参数见§3.1</x:v>
       </x:c>
       <x:c r="AO23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ23" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR23" s="27" t="str">
-        <x:v>能源；效率；多目标组合</x:v>
+        <x:v>群体电量均衡、奖励、任务效率</x:v>
       </x:c>
       <x:c r="AS23" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5750,13 +5750,13 @@
         <x:v>直接：摘要“高峰和低谷时段”“充电策略”“能量均衡”；限制：任务场景给定，未见概率事件模型；3艘实际船舶场景；能量均衡与效率指标</x:v>
       </x:c>
       <x:c r="AV23" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B020 `2.1 算法设计`、`3.1 仿真实验`；B020 `3.1 仿真实验`</x:v>
       </x:c>
       <x:c r="AW23" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX23" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY23" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5765,7 +5765,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA23" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB23" s="27" t="str">
         <x:v>OK</x:v>
@@ -5779,7 +5779,7 @@
         <x:v>L021</x:v>
       </x:c>
       <x:c r="C24" s="27" t="str">
-        <x:v>B021；直接：题名/摘要；改进A；DQN；CBS；数字孪生；限制：随机模型未报告</x:v>
+        <x:v>B021 P2V/V2P、改进A*、DQN、CBS章节；B021 `4.1`–`4.3`</x:v>
       </x:c>
       <x:c r="D24" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -5845,64 +5845,64 @@
         <x:v>路径/任务相邻研究；原分类=混合；动/未报</x:v>
       </x:c>
       <x:c r="Y24" s="27" t="str">
-        <x:v>数字孪生＋改进A*＋DQN＋CBS分层组合</x:v>
+        <x:v>数字孪生路网、AGV状态和预约/冲突信息</x:v>
       </x:c>
       <x:c r="Z24" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>改进A*产生单车路径，DQN决策，CBS协调多车</x:v>
       </x:c>
       <x:c r="AA24" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>CBS检测冲突并添加约束后重规划</x:v>
       </x:c>
       <x:c r="AB24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>无冲突路径集或任务完成</x:v>
       </x:c>
       <x:c r="AC24" s="27" t="str">
-        <x:v>数字孪生＋改进A*＋DQN＋CBS分层组合</x:v>
+        <x:v>P2V采集→A*+DQN路径优化→CBS冲突消解→V2P反馈</x:v>
       </x:c>
       <x:c r="AD24" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>P2V采集→A*+DQN路径优化→CBS冲突消解→V2P反馈</x:v>
       </x:c>
       <x:c r="AE24" s="27" t="str">
-        <x:v>6–12辆AGV；路径和冲突指标</x:v>
+        <x:v>数字孪生无人仓；6–12辆AGV，小/大规模</x:v>
       </x:c>
       <x:c r="AF24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>仓储任务，见算例</x:v>
       </x:c>
       <x:c r="AG24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>6–12</x:v>
       </x:c>
       <x:c r="AJ24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>无人仓数字孪生路网</x:v>
       </x:c>
       <x:c r="AK24" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>小/大规模</x:v>
       </x:c>
       <x:c r="AL24" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>传统A*、DQN/CBS组合及横向方法</x:v>
       </x:c>
       <x:c r="AM24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>路径任务完成；统一训练预算未报告</x:v>
       </x:c>
       <x:c r="AN24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>路径任务完成；统一训练预算未报告</x:v>
       </x:c>
       <x:c r="AO24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ24" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR24" s="27" t="str">
-        <x:v>效率；安全</x:v>
+        <x:v>路径长度、冲突数、规划/运行时间</x:v>
       </x:c>
       <x:c r="AS24" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -5914,13 +5914,13 @@
         <x:v>直接：题名/摘要；改进A；DQN；CBS；数字孪生；限制：随机模型未报告；6–12辆AGV；路径和冲突指标</x:v>
       </x:c>
       <x:c r="AV24" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B021 P2V/V2P、改进A*、DQN、CBS章节；B021 `4.1`–`4.3`</x:v>
       </x:c>
       <x:c r="AW24" s="27" t="str">
         <x:v>随机性/事件生成机制不完整</x:v>
       </x:c>
       <x:c r="AX24" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY24" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -5929,7 +5929,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA24" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB24" s="27" t="str">
         <x:v>OK</x:v>
@@ -5943,7 +5943,7 @@
         <x:v>L022</x:v>
       </x:c>
       <x:c r="C25" s="27" t="str">
-        <x:v>B022；直接：摘要“机床/AGV小车双资源”“数学模型”“工序特征交叉”</x:v>
+        <x:v>B022 `3.1 染色体的编码`、`3.3 算法描述`；B022 `4 仿真结果及分析`</x:v>
       </x:c>
       <x:c r="D25" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -6009,64 +6009,64 @@
         <x:v>核心车间原始研究；原分类=元启发式；静/确</x:v>
       </x:c>
       <x:c r="Y25" s="27" t="str">
-        <x:v>遗传算法＋工序特征交叉；机床/AGV双资源编码</x:v>
+        <x:v>基于工序特征的染色体</x:v>
       </x:c>
       <x:c r="Z25" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>按工序序列同时安排机器与AGV</x:v>
       </x:c>
       <x:c r="AA25" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>交叉变异后按工序优先与双资源约束恢复可行</x:v>
       </x:c>
       <x:c r="AB25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>达到设定代数</x:v>
       </x:c>
       <x:c r="AC25" s="27" t="str">
-        <x:v>遗传算法＋工序特征交叉；机床/AGV双资源编码</x:v>
+        <x:v>初始化→选择→工序特征交叉/变异→评价与替换</x:v>
       </x:c>
       <x:c r="AD25" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>初始化→选择→工序特征交叉/变异→评价与替换</x:v>
       </x:c>
       <x:c r="AE25" s="27" t="str">
-        <x:v>车间算例；具体重复和统计未报告</x:v>
+        <x:v>车间双资源示例算例</x:v>
       </x:c>
       <x:c r="AF25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AG25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AH25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AI25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AJ25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>车间运输路径</x:v>
       </x:c>
       <x:c r="AK25" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>案例</x:v>
       </x:c>
       <x:c r="AL25" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>传统GA/已有结果</x:v>
       </x:c>
       <x:c r="AM25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>算法参数与代数见原文算例段</x:v>
       </x:c>
       <x:c r="AN25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>算法参数与代数见原文算例段</x:v>
       </x:c>
       <x:c r="AO25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ25" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR25" s="27" t="str">
-        <x:v>效率</x:v>
+        <x:v>makespan/求解质量</x:v>
       </x:c>
       <x:c r="AS25" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6078,13 +6078,13 @@
         <x:v>直接：摘要“机床/AGV小车双资源”“数学模型”“工序特征交叉”；车间算例；具体重复和统计未报告</x:v>
       </x:c>
       <x:c r="AV25" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B022 `3.1 染色体的编码`、`3.3 算法描述`；B022 `4 仿真结果及分析`</x:v>
       </x:c>
       <x:c r="AW25" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX25" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY25" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6093,7 +6093,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA25" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB25" s="27" t="str">
         <x:v>OK</x:v>
@@ -6107,7 +6107,7 @@
         <x:v>L023</x:v>
       </x:c>
       <x:c r="C26" s="27" t="str">
-        <x:v>B023；直接：摘要；LS-A3C；Bi-LSTM-CBAM；SUMO/Gazebo；限制：随机模型未报告</x:v>
+        <x:v>B023 `2.1`、`2.2`、第3章；B023 第3章</x:v>
       </x:c>
       <x:c r="D26" s="27" t="str">
         <x:v>Verified</x:v>
@@ -6173,64 +6173,64 @@
         <x:v>路径/任务相邻研究；原分类=学习型；动/未报</x:v>
       </x:c>
       <x:c r="Y26" s="27" t="str">
-        <x:v>LS-A3C＋Bi-LSTM-CBAM；交通信号与路径协同控制</x:v>
+        <x:v>交通信号状态与AGV时序路径特征</x:v>
       </x:c>
       <x:c r="Z26" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>LS-A3C控制信号；Bi-LSTM-CBAM预测/规划路径并推进仿真</x:v>
       </x:c>
       <x:c r="AA26" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>信号相位与路径协同降低冲突/拥堵</x:v>
       </x:c>
       <x:c r="AB26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练收敛/仿真结束</x:v>
       </x:c>
       <x:c r="AC26" s="27" t="str">
-        <x:v>LS-A3C＋Bi-LSTM-CBAM；交通信号与路径协同控制</x:v>
+        <x:v>两模型分别训练后在SUMO/Gazebo协同闭环执行</x:v>
       </x:c>
       <x:c r="AD26" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>两模型分别训练后在SUMO/Gazebo协同闭环执行</x:v>
       </x:c>
       <x:c r="AE26" s="27" t="str">
-        <x:v>SUMO/Gazebo仿真；交通、安全与计算指标</x:v>
+        <x:v>SUMO交通信号与Gazebo多AGV仿真</x:v>
       </x:c>
       <x:c r="AF26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>交通流与AGV路径任务</x:v>
       </x:c>
       <x:c r="AG26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>多AGV，数量见实验</x:v>
       </x:c>
       <x:c r="AJ26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>SUMO/Gazebo路网</x:v>
       </x:c>
       <x:c r="AK26" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>仿真案例</x:v>
       </x:c>
       <x:c r="AL26" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>A3C及无Bi-LSTM/CBAM等对照</x:v>
       </x:c>
       <x:c r="AM26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练参数见§3.1–3.2</x:v>
       </x:c>
       <x:c r="AN26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练参数见§3.1–3.2</x:v>
       </x:c>
       <x:c r="AO26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ26" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR26" s="27" t="str">
-        <x:v>安全；效率；计算成本</x:v>
+        <x:v>等待/通行效率、路径长度、冲突与训练奖励</x:v>
       </x:c>
       <x:c r="AS26" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6242,13 +6242,13 @@
         <x:v>直接：摘要；LS-A3C；Bi-LSTM-CBAM；SUMO/Gazebo；限制：随机模型未报告；SUMO/Gazebo仿真；交通、安全与计算指标</x:v>
       </x:c>
       <x:c r="AV26" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B023 `2.1`、`2.2`、第3章；B023 第3章</x:v>
       </x:c>
       <x:c r="AW26" s="27" t="str">
         <x:v>随机性/事件生成机制不完整</x:v>
       </x:c>
       <x:c r="AX26" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY26" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6257,7 +6257,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA26" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB26" s="27" t="str">
         <x:v>OK</x:v>
@@ -6271,7 +6271,7 @@
         <x:v>L024</x:v>
       </x:c>
       <x:c r="C27" s="27" t="str">
-        <x:v>B024；直接：引言“多周期循环任务指派和全局无碰撞路径规划”“下一周期”；限制：随机模型未报告</x:v>
+        <x:v>B024 `3.4 MA-TA-PPCOA算法流程`、`4.3`；B024 表2–3、`5.1`–`5.2`</x:v>
       </x:c>
       <x:c r="D27" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -6337,64 +6337,64 @@
         <x:v>路径/任务相邻研究；原分类=混合；动/未报</x:v>
       </x:c>
       <x:c r="Y27" s="27" t="str">
-        <x:v>分支切割＋双重优先启发式；在线任务指派与无碰撞路径</x:v>
+        <x:v>任务、AGV、栅格时空路径变量</x:v>
       </x:c>
       <x:c r="Z27" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>双重优先规则指派；五策略改进A*逐车规划三阶段路径</x:v>
       </x:c>
       <x:c r="AA27" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>节点/边冲突检测，等待/重调度后重新规划</x:v>
       </x:c>
       <x:c r="AB27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>所有AGV路径完成；精确法按时限</x:v>
       </x:c>
       <x:c r="AC27" s="27" t="str">
-        <x:v>分支切割＋双重优先启发式；在线任务指派与无碰撞路径</x:v>
+        <x:v>指派→按优先级逐车A*→冲突处理→返回停靠区；Branch-and-cut仅作小规模下界</x:v>
       </x:c>
       <x:c r="AD27" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>指派→按优先级逐车A*→冲突处理→返回停靠区；Branch-and-cut仅作小规模下界</x:v>
       </x:c>
       <x:c r="AE27" s="27" t="str">
-        <x:v>12组及96组实验；下界/gap和秒级决策</x:v>
+        <x:v>12组小规模；144组大规模；5×5至60×60，AGV按规模变化</x:v>
       </x:c>
       <x:c r="AF27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>任务数随实例变化</x:v>
       </x:c>
       <x:c r="AG27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AI27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>随实例变化</x:v>
       </x:c>
       <x:c r="AJ27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>5×5至60×60双向栅格</x:v>
       </x:c>
       <x:c r="AK27" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>12小规模+144大规模</x:v>
       </x:c>
       <x:c r="AL27" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>CPLEX、Branch-and-cut、传统A*及五策略消融</x:v>
       </x:c>
       <x:c r="AM27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>精确法1800/3600/5400秒；启发式要求秒级</x:v>
       </x:c>
       <x:c r="AN27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>精确法1800/3600/5400秒；启发式要求秒级</x:v>
       </x:c>
       <x:c r="AO27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>每组合3例</x:v>
       </x:c>
       <x:c r="AP27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ27" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR27" s="27" t="str">
-        <x:v>效率；安全；计算成本</x:v>
+        <x:v>下界提升、Gap、Obj、求解时间、相对改善</x:v>
       </x:c>
       <x:c r="AS27" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6406,13 +6406,13 @@
         <x:v>直接：引言“多周期循环任务指派和全局无碰撞路径规划”“下一周期”；限制：随机模型未报告；12组及96组实验；下界/gap和秒级决策</x:v>
       </x:c>
       <x:c r="AV27" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B024 `3.4 MA-TA-PPCOA算法流程`、`4.3`；B024 表2–3、`5.1`–`5.2`</x:v>
       </x:c>
       <x:c r="AW27" s="27" t="str">
         <x:v>随机性/事件生成机制不完整</x:v>
       </x:c>
       <x:c r="AX27" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY27" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6421,7 +6421,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA27" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB27" s="27" t="str">
         <x:v>OK</x:v>
@@ -6435,7 +6435,7 @@
         <x:v>L025</x:v>
       </x:c>
       <x:c r="C28" s="27" t="str">
-        <x:v>B025；直接：Abstract；NSGA-II→竞争分配→A→冲突消解调用链</x:v>
+        <x:v>B025 `3.1.1 Encoding and decoding`、`3.2 AGV path search algorithm`；B025 实验章节、Conclusion</x:v>
       </x:c>
       <x:c r="D28" s="27" t="str">
         <x:v>Verified</x:v>
@@ -6501,64 +6501,64 @@
         <x:v>核心车间原始研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y28" s="27" t="str">
-        <x:v>NSGA-II→竞争分配→A*→冲突消解的分层调用链</x:v>
+        <x:v>双资源工序序列/机器与AGV分配</x:v>
       </x:c>
       <x:c r="Z28" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>解码生成机器加工与AGV运输，A*搜索运输路径</x:v>
       </x:c>
       <x:c r="AA28" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>竞争分配与A*规避资源/路径冲突</x:v>
       </x:c>
       <x:c r="AB28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>达到停止预算</x:v>
       </x:c>
       <x:c r="AC28" s="27" t="str">
-        <x:v>NSGA-II→竞争分配→A*→冲突消解的分层调用链</x:v>
+        <x:v>NSGA-II非支配进化；竞争分配与A*嵌入个体解码评价</x:v>
       </x:c>
       <x:c r="AD28" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>NSGA-II非支配进化；竞争分配与A*嵌入个体解码评价</x:v>
       </x:c>
       <x:c r="AE28" s="27" t="str">
-        <x:v>文内算例；可行方案与效率，跨论文只作定性比较</x:v>
+        <x:v>智能制造车间双资源标准算例</x:v>
       </x:c>
       <x:c r="AF28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>标准双资源算例</x:v>
       </x:c>
       <x:c r="AG28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AH28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AI28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见算例</x:v>
       </x:c>
       <x:c r="AJ28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>智能制造车间+A*路网</x:v>
       </x:c>
       <x:c r="AK28" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>标准实例</x:v>
       </x:c>
       <x:c r="AL28" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>NSGA-II/GA类及竞争分配、A*组件对照</x:v>
       </x:c>
       <x:c r="AM28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数和停止见实验章节；当前文本未完整报告重复口径</x:v>
       </x:c>
       <x:c r="AN28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数和停止见实验章节；当前文本未完整报告重复口径</x:v>
       </x:c>
       <x:c r="AO28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ28" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR28" s="27" t="str">
-        <x:v>效率；安全</x:v>
+        <x:v>makespan、AGV运行/路径及多目标解质量</x:v>
       </x:c>
       <x:c r="AS28" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6570,13 +6570,13 @@
         <x:v>直接：Abstract；NSGA-II→竞争分配→A→冲突消解调用链；文内算例；可行方案与效率，跨论文只作定性比较</x:v>
       </x:c>
       <x:c r="AV28" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B025 `3.1.1 Encoding and decoding`、`3.2 AGV path search algorithm`；B025 实验章节、Conclusion</x:v>
       </x:c>
       <x:c r="AW28" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX28" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY28" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6585,7 +6585,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA28" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB28" s="27" t="str">
         <x:v>OK</x:v>
@@ -6599,7 +6599,7 @@
         <x:v>L026</x:v>
       </x:c>
       <x:c r="C29" s="27" t="str">
-        <x:v>B026；直接：Abstract；EAT/SP规则；AGV与场桥集成调度；数值实验</x:v>
+        <x:v>B026 `2 启发式遗传算法`、`2.1编码`；B026 `3.1`–`3.2`</x:v>
       </x:c>
       <x:c r="D29" s="27" t="str">
         <x:v>Original-source verified</x:v>
@@ -6665,64 +6665,64 @@
         <x:v>路径/任务相邻研究；原分类=混合；静/确</x:v>
       </x:c>
       <x:c r="Y29" s="27" t="str">
-        <x:v>EAT/SP规则；AGV与场桥集成调度</x:v>
+        <x:v>双循环码头任务—AGV—场桥分配序列</x:v>
       </x:c>
       <x:c r="Z29" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>EAT规则按最早可用时间派工并生成集成计划</x:v>
       </x:c>
       <x:c r="AA29" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>资源占用约束避免重复分配</x:v>
       </x:c>
       <x:c r="AB29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最大迭代</x:v>
       </x:c>
       <x:c r="AC29" s="27" t="str">
-        <x:v>EAT/SP规则；AGV与场桥集成调度</x:v>
+        <x:v>启发式GA进化，EAT规则嵌入解码/派工</x:v>
       </x:c>
       <x:c r="AD29" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>启发式GA进化，EAT规则嵌入解码/派工</x:v>
       </x:c>
       <x:c r="AE29" s="27" t="str">
-        <x:v>数值实验；均值、最小值、标准差和求解时间</x:v>
+        <x:v>自动化码头双循环AGV–场桥数值算例</x:v>
       </x:c>
       <x:c r="AF29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>码头装卸任务</x:v>
       </x:c>
       <x:c r="AG29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AH29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>场桥</x:v>
       </x:c>
       <x:c r="AI29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>双循环AGV，数量见算例</x:v>
       </x:c>
       <x:c r="AJ29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>自动化码头双循环</x:v>
       </x:c>
       <x:c r="AK29" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>数值案例</x:v>
       </x:c>
       <x:c r="AL29" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>EAT与SP规则</x:v>
       </x:c>
       <x:c r="AM29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>GA参数见§3.1；最大迭代停止</x:v>
       </x:c>
       <x:c r="AN29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>GA参数见§3.1；最大迭代停止</x:v>
       </x:c>
       <x:c r="AO29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ29" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR29" s="27" t="str">
-        <x:v>效率；计算成本</x:v>
+        <x:v>完工/作业时间、mean/min/std、CPU时间</x:v>
       </x:c>
       <x:c r="AS29" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6734,13 +6734,13 @@
         <x:v>直接：Abstract；EAT/SP规则；AGV与场桥集成调度；数值实验；数值实验；均值、最小值、标准差和求解时间</x:v>
       </x:c>
       <x:c r="AV29" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B026 `2 启发式遗传算法`、`2.1编码`；B026 `3.1`–`3.2`</x:v>
       </x:c>
       <x:c r="AW29" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX29" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY29" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6749,7 +6749,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA29" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB29" s="27" t="str">
         <x:v>OK</x:v>
@@ -6763,7 +6763,7 @@
         <x:v>L027</x:v>
       </x:c>
       <x:c r="C30" s="27" t="str">
-        <x:v>B027；直接：Abstract；`AGV scheduling`；决策变量 `M_agv`；新订单和工时变化服从概率分布；限制：动作规则明确选择工序/机器，但是否独立分配AGV不清楚</x:v>
+        <x:v>B027 `MachineRank algorithm`、Algorithms 1–2；B027 `Results and discussion`</x:v>
       </x:c>
       <x:c r="D30" s="27" t="str">
         <x:v>Verified</x:v>
@@ -6829,64 +6829,64 @@
         <x:v>核心车间原始研究；原分类=混合；动/随</x:v>
       </x:c>
       <x:c r="Y30" s="27" t="str">
-        <x:v>MachineRank＋强化学习/D3QN；七种复合调度动作</x:v>
+        <x:v>机器排序分数、车间状态与7个复合规则动作</x:v>
       </x:c>
       <x:c r="Z30" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>MachineRank生成候选机器优先级，D3QN选规则后推进环境</x:v>
       </x:c>
       <x:c r="AA30" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>动作规则保证可执行工序；故障时更新可用机器状态</x:v>
       </x:c>
       <x:c r="AB30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>所有工件完成/训练回合结束</x:v>
       </x:c>
       <x:c r="AC30" s="27" t="str">
-        <x:v>MachineRank＋强化学习/D3QN；七种复合调度动作</x:v>
+        <x:v>MachineRank预处理/排序→D3QN选复合规则→奖励更新网络</x:v>
       </x:c>
       <x:c r="AD30" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>MachineRank预处理/排序→D3QN选复合规则→奖励更新网络</x:v>
       </x:c>
       <x:c r="AE30" s="27" t="str">
-        <x:v>多扰动数值实验；规则和基线对比；概率生成见原文</x:v>
+        <x:v>动态FJSP数值实验，多扰动配置</x:v>
       </x:c>
       <x:c r="AF30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>动态FJSP任务</x:v>
       </x:c>
       <x:c r="AG30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验</x:v>
       </x:c>
       <x:c r="AH30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见实验</x:v>
       </x:c>
       <x:c r="AI30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用/未报告</x:v>
       </x:c>
       <x:c r="AJ30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>柔性车间</x:v>
       </x:c>
       <x:c r="AK30" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多扰动配置</x:v>
       </x:c>
       <x:c r="AL30" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>7个复合规则、MachineRank/D3QN消融及调度规则基线</x:v>
       </x:c>
       <x:c r="AM30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练预算与超参数见Numerical experiments</x:v>
       </x:c>
       <x:c r="AN30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>训练预算与超参数见Numerical experiments</x:v>
       </x:c>
       <x:c r="AO30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ30" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR30" s="27" t="str">
-        <x:v>效率；鲁棒性；多目标组合</x:v>
+        <x:v>makespan、拖期/利用率、奖励与收敛</x:v>
       </x:c>
       <x:c r="AS30" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -6898,13 +6898,13 @@
         <x:v>直接：Abstract；`AGV scheduling`；决策变量 `M_agv`；新订单和工时变化服从概率分布；限制：动作规则明确选择工序/机器，但是否独立分配AGV不清楚；多扰动数值实验；规则和基线对比；概率生成见原文</x:v>
       </x:c>
       <x:c r="AV30" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B027 `MachineRank algorithm`、Algorithms 1–2；B027 `Results and discussion`</x:v>
       </x:c>
       <x:c r="AW30" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX30" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY30" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -6913,7 +6913,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA30" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB30" s="27" t="str">
         <x:v>OK</x:v>
@@ -6927,7 +6927,7 @@
         <x:v>L028</x:v>
       </x:c>
       <x:c r="C31" s="27" t="str">
-        <x:v>B028；直接：Keywords；Introduction；`successive multiple rescheduling`；GA+VNS；限制：未见同时事件模型</x:v>
+        <x:v>B028 `3.1 Encoding and Decoding`、`3.3 Memetic Algorithm`；B028 `4.1`–`4.3`</x:v>
       </x:c>
       <x:c r="D31" s="27" t="str">
         <x:v>Verified</x:v>
@@ -6993,64 +6993,64 @@
         <x:v>核心车间原始研究；原分类=混合；动/确</x:v>
       </x:c>
       <x:c r="Y31" s="27" t="str">
-        <x:v>GA＋VNS模因算法；连续多次重调度</x:v>
+        <x:v>OS–MS–机器人三段编码</x:v>
       </x:c>
       <x:c r="Z31" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>顺序解码机器加工与运输机器人任务</x:v>
       </x:c>
       <x:c r="AA31" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>VNS邻域与事件处理保持工序/资源可行；故障资源不可用</x:v>
       </x:c>
       <x:c r="AB31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最大代数；各重调度窗口结束</x:v>
       </x:c>
       <x:c r="AC31" s="27" t="str">
-        <x:v>GA＋VNS模因算法；连续多次重调度</x:v>
+        <x:v>GA生成子代后嵌入VNS；机器/机器人故障、插单、充电事件触发连续重调度</x:v>
       </x:c>
       <x:c r="AD31" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>GA生成子代后嵌入VNS；机器/机器人故障、插单、充电事件触发连续重调度</x:v>
       </x:c>
       <x:c r="AE31" s="27" t="str">
-        <x:v>EMK等算例；机器/机器人故障、插单和充电的连续重调度</x:v>
+        <x:v>EMK动态联合算例；机器/机器人故障、插单、充电及连续多次重调度</x:v>
       </x:c>
       <x:c r="AF31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>EMK动态任务</x:v>
       </x:c>
       <x:c r="AG31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见EMK实例</x:v>
       </x:c>
       <x:c r="AH31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见EMK实例</x:v>
       </x:c>
       <x:c r="AI31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>运输机器人数量见实例</x:v>
       </x:c>
       <x:c r="AJ31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>EMK运输矩阵</x:v>
       </x:c>
       <x:c r="AK31" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多动态事件</x:v>
       </x:c>
       <x:c r="AL31" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>GA、VNS/模因消融及重调度策略</x:v>
       </x:c>
       <x:c r="AM31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§4.1；代数/重调度窗口停止</x:v>
       </x:c>
       <x:c r="AN31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>参数见§4.1；代数/重调度窗口停止</x:v>
       </x:c>
       <x:c r="AO31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ31" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR31" s="27" t="str">
-        <x:v>效率；稳定性；多目标组合</x:v>
+        <x:v>makespan、重调度表现与稳定性</x:v>
       </x:c>
       <x:c r="AS31" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -7062,13 +7062,13 @@
         <x:v>直接：Keywords；Introduction；`successive multiple rescheduling`；GA+VNS；限制：未见同时事件模型；EMK等算例；机器/机器人故障、插单和充电的连续重调度</x:v>
       </x:c>
       <x:c r="AV31" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B028 `3.1 Encoding and Decoding`、`3.3 Memetic Algorithm`；B028 `4.1`–`4.3`</x:v>
       </x:c>
       <x:c r="AW31" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX31" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY31" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -7077,7 +7077,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA31" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB31" s="27" t="str">
         <x:v>OK</x:v>
@@ -7091,7 +7091,7 @@
         <x:v>L029</x:v>
       </x:c>
       <x:c r="C32" s="27" t="str">
-        <x:v>B029；直接：Abstract；`machine failure interference`；right-shift/complete rescheduling；限制：不含AGV</x:v>
+        <x:v>B029 `2 Genetic algorithm`、`3.2.2 Complete rescheduling`；B029 `4 Results and discussion`</x:v>
       </x:c>
       <x:c r="D32" s="27" t="str">
         <x:v>Verified</x:v>
@@ -7157,64 +7157,64 @@
         <x:v>动态机器相邻研究；原分类=元启发式；动/确</x:v>
       </x:c>
       <x:c r="Y32" s="27" t="str">
-        <x:v>遗传算法；右移与完全重调度</x:v>
+        <x:v>工序序列与机器分配染色体</x:v>
       </x:c>
       <x:c r="Z32" s="27" t="str">
-        <x:v>待N5逐篇拆分解码/环境转移</x:v>
+        <x:v>解码初始FJSP及故障后的剩余工序</x:v>
       </x:c>
       <x:c r="AA32" s="27" t="str">
-        <x:v>待N5逐篇拆分修复/冲突处理</x:v>
+        <x:v>右移保持分配顺序；完全重调度对未开工部分重新编码求解</x:v>
       </x:c>
       <x:c r="AB32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>最大代数/重调度完成</x:v>
       </x:c>
       <x:c r="AC32" s="27" t="str">
-        <x:v>遗传算法；右移与完全重调度</x:v>
+        <x:v>GA求初始计划；机器故障后分别执行右移或完全重调度</x:v>
       </x:c>
       <x:c r="AD32" s="27" t="str">
-        <x:v>见算法名称与职责；具体插入点待N5抽取</x:v>
+        <x:v>GA求初始计划；机器故障后分别执行右移或完全重调度</x:v>
       </x:c>
       <x:c r="AE32" s="27" t="str">
-        <x:v>机器故障算例；延误率；右移与完全重调度比较</x:v>
+        <x:v>Brandimarte mk系列机器故障重调度算例</x:v>
       </x:c>
       <x:c r="AF32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>Brandimarte mk系列</x:v>
       </x:c>
       <x:c r="AG32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见mk实例</x:v>
       </x:c>
       <x:c r="AH32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>见mk实例</x:v>
       </x:c>
       <x:c r="AI32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="AJ32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>柔性车间</x:v>
       </x:c>
       <x:c r="AK32" s="27" t="str">
-        <x:v>待N6分级</x:v>
+        <x:v>多机器故障案例</x:v>
       </x:c>
       <x:c r="AL32" s="27" t="str">
-        <x:v>见文内对照；待N6标准化</x:v>
+        <x:v>右移与完全重调度</x:v>
       </x:c>
       <x:c r="AM32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>GA参数/停止见实验设置</x:v>
       </x:c>
       <x:c r="AN32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>GA参数/停止见实验设置</x:v>
       </x:c>
       <x:c r="AO32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AP32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AQ32" s="27" t="str">
-        <x:v>待N6抽取</x:v>
+        <x:v>未报告</x:v>
       </x:c>
       <x:c r="AR32" s="27" t="str">
-        <x:v>效率；稳定性</x:v>
+        <x:v>makespan、平均延误率、求解时间</x:v>
       </x:c>
       <x:c r="AS32" s="27" t="str">
         <x:v>原始Markdown与N2/N4派生证据可用</x:v>
@@ -7226,13 +7226,13 @@
         <x:v>直接：Abstract；`machine failure interference`；right-shift/complete rescheduling；限制：不含AGV；机器故障算例；延误率；右移与完全重调度比较</x:v>
       </x:c>
       <x:c r="AV32" s="27" t="str">
-        <x:v>泛式分类仅用于全景整理，不构成当前静态创新性判断</x:v>
+        <x:v>N5/N6深度抽取：B029 `2 Genetic algorithm`、`3.2.2 Complete rescheduling`；B029 `4 Results and discussion`</x:v>
       </x:c>
       <x:c r="AW32" s="27" t="str">
         <x:v>跨论文性能不可直接比较</x:v>
       </x:c>
       <x:c r="AX32" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>深度抽取完成；原文未报告项已显式保留，不得补猜</x:v>
       </x:c>
       <x:c r="AY32" s="27" t="str">
         <x:v>direct evidence</x:v>
@@ -7241,7 +7241,7 @@
         <x:v>direct</x:v>
       </x:c>
       <x:c r="BA32" s="27" t="str">
-        <x:v>First-pass complete</x:v>
+        <x:v>Deep extraction complete</x:v>
       </x:c>
       <x:c r="BB32" s="27" t="str">
         <x:v>OK</x:v>
@@ -7286,7 +7286,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda75840bcc854de8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eec9a943ceb40b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7610,7 +7610,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21ae9da8df44230"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2047ca457424345"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8084,7 +8084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9ae27d360444d6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f9fdb95d40f4d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8189,19 +8189,19 @@
       </x:c>
       <x:c r="D4" s="27"/>
       <x:c r="E4" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F4" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G4" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H4" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I4" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J4" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8225,19 +8225,19 @@
       </x:c>
       <x:c r="D5" s="27"/>
       <x:c r="E5" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G5" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H5" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I5" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J5" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8261,19 +8261,19 @@
       </x:c>
       <x:c r="D6" s="27"/>
       <x:c r="E6" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G6" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H6" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I6" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J6" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8297,19 +8297,19 @@
       </x:c>
       <x:c r="D7" s="27"/>
       <x:c r="E7" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F7" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G7" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H7" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I7" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J7" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8333,19 +8333,19 @@
       </x:c>
       <x:c r="D8" s="27"/>
       <x:c r="E8" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F8" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G8" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H8" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J8" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8369,19 +8369,19 @@
       </x:c>
       <x:c r="D9" s="27"/>
       <x:c r="E9" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F9" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G9" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H9" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I9" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J9" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8405,19 +8405,19 @@
       </x:c>
       <x:c r="D10" s="27"/>
       <x:c r="E10" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F10" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G10" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H10" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I10" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J10" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8441,19 +8441,19 @@
       </x:c>
       <x:c r="D11" s="27"/>
       <x:c r="E11" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F11" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G11" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H11" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I11" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J11" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8477,19 +8477,19 @@
       </x:c>
       <x:c r="D12" s="27"/>
       <x:c r="E12" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F12" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G12" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H12" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I12" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J12" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8513,19 +8513,19 @@
       </x:c>
       <x:c r="D13" s="27"/>
       <x:c r="E13" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F13" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G13" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H13" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I13" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J13" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8549,19 +8549,19 @@
       </x:c>
       <x:c r="D14" s="27"/>
       <x:c r="E14" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F14" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G14" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H14" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I14" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J14" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8585,19 +8585,19 @@
       </x:c>
       <x:c r="D15" s="27"/>
       <x:c r="E15" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F15" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H15" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I15" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J15" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8621,19 +8621,19 @@
       </x:c>
       <x:c r="D16" s="27"/>
       <x:c r="E16" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F16" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G16" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H16" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I16" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J16" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8657,19 +8657,19 @@
       </x:c>
       <x:c r="D17" s="27"/>
       <x:c r="E17" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F17" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G17" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H17" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I17" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J17" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8693,19 +8693,19 @@
       </x:c>
       <x:c r="D18" s="27"/>
       <x:c r="E18" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F18" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G18" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H18" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I18" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J18" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8729,19 +8729,19 @@
       </x:c>
       <x:c r="D19" s="27"/>
       <x:c r="E19" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F19" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G19" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H19" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I19" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J19" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8765,19 +8765,19 @@
       </x:c>
       <x:c r="D20" s="27"/>
       <x:c r="E20" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F20" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G20" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H20" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I20" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J20" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8801,19 +8801,19 @@
       </x:c>
       <x:c r="D21" s="27"/>
       <x:c r="E21" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F21" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G21" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H21" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I21" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J21" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8837,19 +8837,19 @@
       </x:c>
       <x:c r="D22" s="27"/>
       <x:c r="E22" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F22" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G22" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H22" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I22" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J22" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8873,19 +8873,19 @@
       </x:c>
       <x:c r="D23" s="27"/>
       <x:c r="E23" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F23" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G23" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H23" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I23" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J23" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8909,19 +8909,19 @@
       </x:c>
       <x:c r="D24" s="27"/>
       <x:c r="E24" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F24" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G24" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H24" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I24" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J24" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8945,19 +8945,19 @@
       </x:c>
       <x:c r="D25" s="27"/>
       <x:c r="E25" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F25" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G25" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H25" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I25" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J25" s="27" t="str">
         <x:v>Codex</x:v>
@@ -8981,19 +8981,19 @@
       </x:c>
       <x:c r="D26" s="27"/>
       <x:c r="E26" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F26" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G26" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H26" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I26" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J26" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9017,19 +9017,19 @@
       </x:c>
       <x:c r="D27" s="27"/>
       <x:c r="E27" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F27" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G27" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H27" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I27" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J27" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9053,19 +9053,19 @@
       </x:c>
       <x:c r="D28" s="27"/>
       <x:c r="E28" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F28" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G28" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H28" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I28" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J28" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9089,19 +9089,19 @@
       </x:c>
       <x:c r="D29" s="27"/>
       <x:c r="E29" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F29" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G29" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H29" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I29" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J29" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9125,19 +9125,19 @@
       </x:c>
       <x:c r="D30" s="27"/>
       <x:c r="E30" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F30" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G30" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H30" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I30" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J30" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9161,19 +9161,19 @@
       </x:c>
       <x:c r="D31" s="27"/>
       <x:c r="E31" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F31" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G31" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H31" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I31" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J31" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9197,19 +9197,19 @@
       </x:c>
       <x:c r="D32" s="27"/>
       <x:c r="E32" s="27" t="str">
-        <x:v>算法组件已完成首轮登记；编码/解码、完整预算、重复、种子和统计字段仍须N5/N6原文精读</x:v>
+        <x:v>N5/N6逐篇抽取已完成；随机种子未报告；统计检验未报告；缺失项按原文保留</x:v>
       </x:c>
       <x:c r="F32" s="27" t="str">
         <x:v>影响算法模块归因和跨论文可比性</x:v>
       </x:c>
       <x:c r="G32" s="27" t="str">
-        <x:v>N5抽取算法调用链；N6抽取实验协议</x:v>
+        <x:v>已回填Evidence；缺失信息标为未报告/不适用，不再作为待抽取项</x:v>
       </x:c>
       <x:c r="H32" s="27" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="I32" s="27" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="J32" s="27" t="str">
         <x:v>Codex</x:v>
@@ -9236,7 +9236,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe4a9fc6c78f43e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3af9c9399647f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9322,14 +9322,26 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="42"/>
-      <x:c r="B5" s="31"/>
-      <x:c r="C5" s="29"/>
-      <x:c r="D5" s="29"/>
-      <x:c r="E5" s="29"/>
-      <x:c r="F5" s="29"/>
+      <x:c r="A5" s="42" t="str">
+        <x:v>v0.2</x:v>
+      </x:c>
+      <x:c r="B5" s="31" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="C5" s="29" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D5" s="29" t="str">
+        <x:v>完成L001–L029的N5算法调用链与N6实验协议深度抽取；缺失信息显式标注未报告/不适用</x:v>
+      </x:c>
+      <x:c r="E5" s="29" t="str">
+        <x:v>B001–B029原文转换文本；P02_N5N6逐篇深度抽取.md</x:v>
+      </x:c>
+      <x:c r="F5" s="29" t="str">
+        <x:v>Deep extraction complete</x:v>
+      </x:c>
       <x:c r="G5" s="41" t="str">
-        <x:f>IF(COUNTA(B5:F5)=0,"",IF(A5="","MISSING ID","OK"))</x:f>
+        <x:v>OK</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9540,6 +9552,15 @@
       <x:c r="G24" s="46" t="str">
         <x:f>IF(COUNTA(B24:F24)=0,"",IF(A24="","MISSING ID","OK"))</x:f>
       </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9553,7 +9574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5700f1fa2d9243c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04ca5b85c76842d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>